<commit_message>
Study the existing data
</commit_message>
<xml_diff>
--- a/data/raw/Basic Course Score.xlsx
+++ b/data/raw/Basic Course Score.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Projects\kshrd-basic-course-student-performance-analytics\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827691E4-3A34-416F-AA9E-A2934EDFD93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E8C18A-C460-418F-9819-67C766C65F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="March" sheetId="1" r:id="rId1"/>
@@ -3351,10 +3351,7 @@
       <c r="M58" s="7"/>
       <c r="N58" s="7"/>
       <c r="O58" s="7"/>
-      <c r="P58" s="6">
-        <f>SUM(P2:P57)</f>
-        <v>3256.5</v>
-      </c>
+      <c r="P58" s="6"/>
     </row>
     <row r="59" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
       <c r="J59" s="7"/>
@@ -14775,10 +14772,7 @@
       </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="Q57" s="6">
-        <f>SUM(Q1:Q56)</f>
-        <v>3038.5</v>
-      </c>
+      <c r="Q57" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17542,10 +17536,7 @@
       <c r="M56" s="7"/>
       <c r="N56" s="7"/>
       <c r="O56" s="7"/>
-      <c r="P56" s="6">
-        <f>SUM(P2:P55)</f>
-        <v>4677.5</v>
-      </c>
+      <c r="P56" s="6"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="J57" s="7"/>
@@ -28373,10 +28364,7 @@
       <c r="K55" s="7"/>
       <c r="L55" s="7"/>
       <c r="M55" s="7"/>
-      <c r="N55" s="6">
-        <f>SUM(N1:N54)</f>
-        <v>5299</v>
-      </c>
+      <c r="N55" s="6"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="I56" s="7"/>

</xml_diff>